<commit_message>
Mise à jour des profils FHIR Suite aux issues remontés (#162)
* Mise à jour des profils suite aux issues

* Mise à jour des profils FHIR suite issues NRISS 13cce64d85c5eaf8e78427aa2e48b6c0e62b235b
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-fr-imaging-study-document.xlsx
+++ b/main/ig/StructureDefinition-fr-imaging-study-document.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-16T14:27:29+00:00</t>
+    <t>2026-06-18T14:40:49+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -797,7 +797,7 @@
 </t>
   </si>
   <si>
-    <t>Number of Study Related Series</t>
+    <t>Nombre de séries</t>
   </si>
   <si>
     <t>Number of Series in the Study. This value given may be larger than the number of series elements this Resource contains due to resource availability, security, or other factors. This element should be present if any series elements are present.</t>
@@ -4384,7 +4384,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="23" hidden="true">
+    <row r="23">
       <c r="A23" t="s" s="2">
         <v>245</v>
       </c>
@@ -4403,7 +4403,7 @@
         <v>89</v>
       </c>
       <c r="H23" t="s" s="2">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="I23" t="s" s="2">
         <v>78</v>

</xml_diff>